<commit_message>
Add RICE prioritization (workbook sheet + app tab + docs)
- Планирование_спринта_PRO.xlsx: new «RICE» sheet — features scored by
  RICE = (Reach × Impact × Confidence) / Effort with formulas, dropdowns
  (Impact/Confidence), RAG priority, color-scale on score, ranking, and a
  bar chart. Now 29 sheets.
- index.html: «RICE» tab — editable inputs, auto RICE score / rank /
  priority (RAG), bar chart, and a methodology legend. Added to Excel
  export; Reset now runs migrate() so new collections survive a reset.
- data/seed.json: RICE dataset (10 features).
- Both description docs: RICE section (methodology + parameters table);
  illustrated doc also gets a RICE bar chart image.
- README: note the RICE feature.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Планирование_спринта_PRO.xlsx
+++ b/Планирование_спринта_PRO.xlsx
@@ -11,29 +11,30 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Параметры" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Дорожная карта" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Кварталы" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Квартальный roadmap" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Релизы" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Вехи" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Технический долг" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ретроспективы" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Бюджет" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OKR" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ёмкость на горизонт" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Гант" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Капасити" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Календарь" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Загрузка по ролям" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Бэклог" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сгорание" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Качество" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Баги" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CFD" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Метрики и прогноз" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cycle time" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Риски" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Матрица рисков" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Распределение" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Time to Market" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RICE" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Квартальный roadmap" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Релизы" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Вехи" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Технический долг" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ретроспективы" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Бюджет" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OKR" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ёмкость на горизонт" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Гант" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Капасити" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Календарь" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Загрузка по ролям" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Бэклог" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сгорание" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Качество" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Баги" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CFD" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Метрики и прогноз" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cycle time" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Риски" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Матрица рисков" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Распределение" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Time to Market" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -42,14 +43,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="dd\.mm"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
     <numFmt numFmtId="168" formatCode="dd\.mm\.yy"/>
+    <numFmt numFmtId="169" formatCode="# ##0"/>
+    <numFmt numFmtId="170" formatCode="# ##0.0"/>
   </numFmts>
-  <fonts count="50">
+  <fonts count="53">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -339,6 +342,21 @@
       <color rgb="FF1F4E78"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="FF5A6B82"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="51">
     <fill>
@@ -593,7 +611,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -839,11 +857,25 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="229">
+  <cellXfs count="240">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1399,11 +1431,30 @@
     <xf numFmtId="167" fontId="16" fillId="50" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="48" fillId="48" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="4" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="39">
+  <dxfs count="42">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1674,6 +1725,27 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF8D7DA"/>
         </patternFill>
       </fill>
     </dxf>
@@ -13434,6 +13506,87 @@
       <tx>
         <rich>
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>RICE score по фичам</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'RICE'!G4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'RICE'!$B$5:$B$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'RICE'!$G$5:$G$14</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart44.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
@@ -13854,7 +14007,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart44.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart45.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -14151,7 +14304,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart46.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -14285,7 +14438,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart47.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -14436,7 +14589,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart48.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -14575,7 +14728,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart49.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -15001,201 +15154,6 @@
       <legendPos val="b"/>
       <overlay val="0"/>
     </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart49.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="ru-RU"/>
-              <a:t>Расход бюджета (накопл.)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-      <overlay val="0"/>
-    </title>
-    <plotArea>
-      <layout/>
-      <lineChart>
-        <grouping val="standard"/>
-        <varyColors val="1"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>Бюджет!$D$6</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>Накопл. стоимость (₽)</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
-              <a:solidFill>
-                <a:srgbClr val="C00000"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>Бюджет!$A$7:$A$17</f>
-              <numCache>
-                <formatCode>General</formatCode>
-                <ptCount val="11"/>
-                <pt idx="0">
-                  <v>1</v>
-                </pt>
-                <pt idx="1">
-                  <v>2</v>
-                </pt>
-                <pt idx="2">
-                  <v>3</v>
-                </pt>
-                <pt idx="3">
-                  <v>4</v>
-                </pt>
-                <pt idx="4">
-                  <v>5</v>
-                </pt>
-                <pt idx="5">
-                  <v>6</v>
-                </pt>
-                <pt idx="6">
-                  <v>7</v>
-                </pt>
-                <pt idx="7">
-                  <v>8</v>
-                </pt>
-                <pt idx="8">
-                  <v>9</v>
-                </pt>
-                <pt idx="9">
-                  <v>10</v>
-                </pt>
-                <pt idx="10">
-                  <v>11</v>
-                </pt>
-              </numCache>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>Бюджет!$D$7:$D$17</f>
-              <numCache>
-                <formatCode>#,##0</formatCode>
-                <ptCount val="11"/>
-                <pt idx="0">
-                  <v>742400.0000000001</v>
-                </pt>
-                <pt idx="1">
-                  <v>1504000</v>
-                </pt>
-                <pt idx="2">
-                  <v>2265600</v>
-                </pt>
-                <pt idx="3">
-                  <v>3027200</v>
-                </pt>
-                <pt idx="4">
-                  <v>3772800</v>
-                </pt>
-                <pt idx="5">
-                  <v>4534400</v>
-                </pt>
-                <pt idx="6">
-                  <v>5219840</v>
-                </pt>
-                <pt idx="7">
-                  <v>5949440</v>
-                </pt>
-                <pt idx="8">
-                  <v>6711040</v>
-                </pt>
-                <pt idx="9">
-                  <v>7472640</v>
-                </pt>
-                <pt idx="10">
-                  <v>8158080</v>
-                </pt>
-              </numCache>
-            </numRef>
-          </val>
-          <smooth val="1"/>
-        </ser>
-        <dLbls>
-          <showLegendKey val="0"/>
-          <showVal val="0"/>
-          <showCatName val="0"/>
-          <showSerName val="0"/>
-          <showPercent val="0"/>
-          <showBubbleSize val="0"/>
-        </dLbls>
-        <smooth val="0"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="b"/>
-        <numFmt formatCode="General" sourceLinked="1"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <crossAx val="100"/>
-        <crosses val="autoZero"/>
-        <auto val="1"/>
-        <lblAlgn val="ctr"/>
-        <lblOffset val="100"/>
-        <noMultiLvlLbl val="1"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <numFmt formatCode="#,##0" sourceLinked="1"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <crossAx val="10"/>
-        <crosses val="autoZero"/>
-        <crossBetween val="between"/>
-      </valAx>
-    </plotArea>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -15807,6 +15765,201 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="ru-RU"/>
+              <a:t>Расход бюджета (накопл.)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+      <overlay val="0"/>
+    </title>
+    <plotArea>
+      <layout/>
+      <lineChart>
+        <grouping val="standard"/>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>Бюджет!$D$6</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v>Накопл. стоимость (₽)</v>
+                </pt>
+              </strCache>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>Бюджет!$A$7:$A$17</f>
+              <numCache>
+                <formatCode>General</formatCode>
+                <ptCount val="11"/>
+                <pt idx="0">
+                  <v>1</v>
+                </pt>
+                <pt idx="1">
+                  <v>2</v>
+                </pt>
+                <pt idx="2">
+                  <v>3</v>
+                </pt>
+                <pt idx="3">
+                  <v>4</v>
+                </pt>
+                <pt idx="4">
+                  <v>5</v>
+                </pt>
+                <pt idx="5">
+                  <v>6</v>
+                </pt>
+                <pt idx="6">
+                  <v>7</v>
+                </pt>
+                <pt idx="7">
+                  <v>8</v>
+                </pt>
+                <pt idx="8">
+                  <v>9</v>
+                </pt>
+                <pt idx="9">
+                  <v>10</v>
+                </pt>
+                <pt idx="10">
+                  <v>11</v>
+                </pt>
+              </numCache>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>Бюджет!$D$7:$D$17</f>
+              <numCache>
+                <formatCode>#,##0</formatCode>
+                <ptCount val="11"/>
+                <pt idx="0">
+                  <v>742400.0000000001</v>
+                </pt>
+                <pt idx="1">
+                  <v>1504000</v>
+                </pt>
+                <pt idx="2">
+                  <v>2265600</v>
+                </pt>
+                <pt idx="3">
+                  <v>3027200</v>
+                </pt>
+                <pt idx="4">
+                  <v>3772800</v>
+                </pt>
+                <pt idx="5">
+                  <v>4534400</v>
+                </pt>
+                <pt idx="6">
+                  <v>5219840</v>
+                </pt>
+                <pt idx="7">
+                  <v>5949440</v>
+                </pt>
+                <pt idx="8">
+                  <v>6711040</v>
+                </pt>
+                <pt idx="9">
+                  <v>7472640</v>
+                </pt>
+                <pt idx="10">
+                  <v>8158080</v>
+                </pt>
+              </numCache>
+            </numRef>
+          </val>
+          <smooth val="1"/>
+        </ser>
+        <dLbls>
+          <showLegendKey val="0"/>
+          <showVal val="0"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="0"/>
+          <showBubbleSize val="0"/>
+        </dLbls>
+        <smooth val="0"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="b"/>
+        <numFmt formatCode="General" sourceLinked="1"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <crossAx val="100"/>
+        <crosses val="autoZero"/>
+        <auto val="1"/>
+        <lblAlgn val="ctr"/>
+        <lblOffset val="100"/>
+        <noMultiLvlLbl val="1"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <numFmt formatCode="#,##0" sourceLinked="1"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <crossAx val="10"/>
+        <crosses val="autoZero"/>
+        <crossBetween val="between"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart51.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="ru-RU"/>
               <a:t xml:space="preserve">Прогресс </a:t>
             </a:r>
             <a:r>
@@ -15948,7 +16101,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart51.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart52.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -16158,7 +16311,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart52.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart53.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -16954,7 +17107,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart53.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart54.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -17252,7 +17405,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart54.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart55.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -17626,7 +17779,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart55.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart56.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -18010,7 +18163,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart56.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart57.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -18368,7 +18521,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart57.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart58.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -18669,7 +18822,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart58.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart59.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -18852,162 +19005,6 @@
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart59.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="ru-RU"/>
-              <a:t>Доля багов по спринтам</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-      <overlay val="1"/>
-    </title>
-    <plotArea>
-      <layout/>
-      <pieChart>
-        <varyColors val="1"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <dLbls>
-            <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-            <showLegendKey val="0"/>
-            <showVal val="0"/>
-            <showCatName val="0"/>
-            <showSerName val="0"/>
-            <showPercent val="1"/>
-            <showBubbleSize val="1"/>
-            <showLeaderLines val="1"/>
-          </dLbls>
-          <cat>
-            <numRef>
-              <f>Баги!$J$6:$J$16</f>
-              <numCache>
-                <formatCode>General</formatCode>
-                <ptCount val="11"/>
-                <pt idx="0">
-                  <v>1</v>
-                </pt>
-                <pt idx="1">
-                  <v>2</v>
-                </pt>
-                <pt idx="2">
-                  <v>3</v>
-                </pt>
-                <pt idx="3">
-                  <v>4</v>
-                </pt>
-                <pt idx="4">
-                  <v>5</v>
-                </pt>
-                <pt idx="5">
-                  <v>6</v>
-                </pt>
-                <pt idx="6">
-                  <v>7</v>
-                </pt>
-                <pt idx="7">
-                  <v>8</v>
-                </pt>
-                <pt idx="8">
-                  <v>9</v>
-                </pt>
-                <pt idx="9">
-                  <v>10</v>
-                </pt>
-                <pt idx="10">
-                  <v>11</v>
-                </pt>
-              </numCache>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>Баги!$P$6:$P$16</f>
-              <numCache>
-                <formatCode>General</formatCode>
-                <ptCount val="11"/>
-                <pt idx="0">
-                  <v>5</v>
-                </pt>
-                <pt idx="1">
-                  <v>6</v>
-                </pt>
-                <pt idx="2">
-                  <v>2</v>
-                </pt>
-                <pt idx="3">
-                  <v>#N/A</v>
-                </pt>
-                <pt idx="4">
-                  <v>#N/A</v>
-                </pt>
-                <pt idx="5">
-                  <v>#N/A</v>
-                </pt>
-                <pt idx="6">
-                  <v>#N/A</v>
-                </pt>
-                <pt idx="7">
-                  <v>#N/A</v>
-                </pt>
-                <pt idx="8">
-                  <v>#N/A</v>
-                </pt>
-                <pt idx="9">
-                  <v>#N/A</v>
-                </pt>
-                <pt idx="10">
-                  <v>#N/A</v>
-                </pt>
-              </numCache>
-            </numRef>
-          </val>
-        </ser>
-        <dLbls>
-          <showLegendKey val="0"/>
-          <showVal val="0"/>
-          <showCatName val="0"/>
-          <showSerName val="0"/>
-          <showPercent val="1"/>
-          <showBubbleSize val="1"/>
-          <showLeaderLines val="1"/>
-        </dLbls>
-        <firstSliceAng val="0"/>
-      </pieChart>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-      <overlay val="0"/>
-    </legend>
-    <plotVisOnly val="0"/>
     <dispBlanksAs val="gap"/>
   </chart>
 </chartSpace>
@@ -19278,6 +19275,162 @@
 </file>
 
 <file path=xl/charts/chart60.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="ru-RU"/>
+              <a:t>Доля багов по спринтам</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+      <overlay val="1"/>
+    </title>
+    <plotArea>
+      <layout/>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <dLbls>
+            <spPr>
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="1"/>
+            <showBubbleSize val="1"/>
+            <showLeaderLines val="1"/>
+          </dLbls>
+          <cat>
+            <numRef>
+              <f>Баги!$J$6:$J$16</f>
+              <numCache>
+                <formatCode>General</formatCode>
+                <ptCount val="11"/>
+                <pt idx="0">
+                  <v>1</v>
+                </pt>
+                <pt idx="1">
+                  <v>2</v>
+                </pt>
+                <pt idx="2">
+                  <v>3</v>
+                </pt>
+                <pt idx="3">
+                  <v>4</v>
+                </pt>
+                <pt idx="4">
+                  <v>5</v>
+                </pt>
+                <pt idx="5">
+                  <v>6</v>
+                </pt>
+                <pt idx="6">
+                  <v>7</v>
+                </pt>
+                <pt idx="7">
+                  <v>8</v>
+                </pt>
+                <pt idx="8">
+                  <v>9</v>
+                </pt>
+                <pt idx="9">
+                  <v>10</v>
+                </pt>
+                <pt idx="10">
+                  <v>11</v>
+                </pt>
+              </numCache>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>Баги!$P$6:$P$16</f>
+              <numCache>
+                <formatCode>General</formatCode>
+                <ptCount val="11"/>
+                <pt idx="0">
+                  <v>5</v>
+                </pt>
+                <pt idx="1">
+                  <v>6</v>
+                </pt>
+                <pt idx="2">
+                  <v>2</v>
+                </pt>
+                <pt idx="3">
+                  <v>#N/A</v>
+                </pt>
+                <pt idx="4">
+                  <v>#N/A</v>
+                </pt>
+                <pt idx="5">
+                  <v>#N/A</v>
+                </pt>
+                <pt idx="6">
+                  <v>#N/A</v>
+                </pt>
+                <pt idx="7">
+                  <v>#N/A</v>
+                </pt>
+                <pt idx="8">
+                  <v>#N/A</v>
+                </pt>
+                <pt idx="9">
+                  <v>#N/A</v>
+                </pt>
+                <pt idx="10">
+                  <v>#N/A</v>
+                </pt>
+              </numCache>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showLegendKey val="0"/>
+          <showVal val="0"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="1"/>
+          <showBubbleSize val="1"/>
+          <showLeaderLines val="1"/>
+        </dLbls>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+      <overlay val="0"/>
+    </legend>
+    <plotVisOnly val="0"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart61.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -19738,7 +19891,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart61.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart62.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -19935,7 +20088,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart62.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart63.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -20127,7 +20280,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart63.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart64.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -20379,7 +20532,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart64.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart65.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -20631,7 +20784,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart65.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart66.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -20950,7 +21103,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart66.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart67.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -21715,7 +21868,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart67.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart68.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -21916,7 +22069,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart68.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart69.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -22061,7 +22214,147 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart69.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="ru-RU"/>
+              <a:t>% выполнения по кварталам</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+      <overlay val="0"/>
+    </title>
+    <plotArea>
+      <layout/>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>Кварталы!$G$4</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v>% выпол-
+нения</v>
+                </pt>
+              </strCache>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="70AD47"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <invertIfNegative val="1"/>
+          <cat>
+            <strRef>
+              <f>Кварталы!$A$5:$A$7</f>
+              <strCache>
+                <ptCount val="3"/>
+                <pt idx="0">
+                  <v>Q3 2026</v>
+                </pt>
+                <pt idx="1">
+                  <v>Q4 2026</v>
+                </pt>
+                <pt idx="2">
+                  <v>Q1 2027</v>
+                </pt>
+              </strCache>
+            </strRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>Кварталы!$G$5:$G$7</f>
+              <numCache>
+                <formatCode>0%</formatCode>
+                <ptCount val="3"/>
+                <pt idx="0">
+                  <v>0.3551401869158878</v>
+                </pt>
+                <pt idx="1">
+                  <v>0</v>
+                </pt>
+                <pt idx="2">
+                  <v>0</v>
+                </pt>
+              </numCache>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showLegendKey val="0"/>
+          <showVal val="0"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="0"/>
+          <showBubbleSize val="0"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="b"/>
+        <numFmt formatCode="General" sourceLinked="1"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <crossAx val="100"/>
+        <crosses val="autoZero"/>
+        <auto val="1"/>
+        <lblAlgn val="ctr"/>
+        <lblOffset val="100"/>
+        <noMultiLvlLbl val="1"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <numFmt formatCode="0%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <crossAx val="10"/>
+        <crosses val="autoZero"/>
+        <crossBetween val="between"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart70.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -22294,147 +22587,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="ru-RU"/>
-              <a:t>% выполнения по кварталам</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-      <overlay val="0"/>
-    </title>
-    <plotArea>
-      <layout/>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <varyColors val="1"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>Кварталы!$G$4</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>% выпол-
-нения</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="70AD47"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <invertIfNegative val="1"/>
-          <cat>
-            <strRef>
-              <f>Кварталы!$A$5:$A$7</f>
-              <strCache>
-                <ptCount val="3"/>
-                <pt idx="0">
-                  <v>Q3 2026</v>
-                </pt>
-                <pt idx="1">
-                  <v>Q4 2026</v>
-                </pt>
-                <pt idx="2">
-                  <v>Q1 2027</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>Кварталы!$G$5:$G$7</f>
-              <numCache>
-                <formatCode>0%</formatCode>
-                <ptCount val="3"/>
-                <pt idx="0">
-                  <v>0.3551401869158878</v>
-                </pt>
-                <pt idx="1">
-                  <v>0</v>
-                </pt>
-                <pt idx="2">
-                  <v>0</v>
-                </pt>
-              </numCache>
-            </numRef>
-          </val>
-        </ser>
-        <dLbls>
-          <showLegendKey val="0"/>
-          <showVal val="0"/>
-          <showCatName val="0"/>
-          <showSerName val="0"/>
-          <showPercent val="0"/>
-          <showBubbleSize val="0"/>
-        </dLbls>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="b"/>
-        <numFmt formatCode="General" sourceLinked="1"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <crossAx val="100"/>
-        <crosses val="autoZero"/>
-        <auto val="1"/>
-        <lblAlgn val="ctr"/>
-        <lblOffset val="100"/>
-        <noMultiLvlLbl val="1"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <numFmt formatCode="0%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <crossAx val="10"/>
-        <crosses val="autoZero"/>
-        <crossBetween val="between"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart70.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart71.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -24402,6 +24555,33 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6120000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
       <col>8</col>
       <colOff>0</colOff>
       <row>3</row>
@@ -24425,7 +24605,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -24452,7 +24632,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -24479,7 +24659,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing14.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -24506,7 +24686,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing15.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -24555,7 +24735,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing16.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -24582,7 +24762,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing17.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -24653,7 +24833,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing18.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -24680,7 +24860,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing19.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -24795,33 +24975,6 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing19.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>541020</colOff>
-      <row>9</row>
-      <rowOff>38100</rowOff>
-    </from>
-    <ext cx="7920000" cy="3240000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -24875,6 +25028,33 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
+      <col>5</col>
+      <colOff>541020</colOff>
+      <row>9</row>
+      <rowOff>38100</rowOff>
+    </from>
+    <ext cx="7920000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing21.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
       <col>10</col>
       <colOff>0</colOff>
       <row>3</row>
@@ -24898,7 +25078,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing22.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -24955,7 +25135,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing23.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -24982,7 +25162,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing24.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -25133,6 +25313,33 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6120000" cy="3060000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
       <col>6</col>
       <colOff>0</colOff>
       <row>3</row>
@@ -25156,7 +25363,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -25183,7 +25390,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -25210,7 +25417,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -25273,33 +25480,6 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>7</col>
-      <colOff>0</colOff>
-      <row>5</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="6120000" cy="2880000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -25845,6 +26025,771 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="16.6640625" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="10.77734375" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="17.4" customHeight="1">
+      <c r="A1" s="198" t="inlineStr">
+        <is>
+          <t>Технический долг</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="199" t="inlineStr">
+        <is>
+          <t>Реестр техдолга: область, тип, влияние, оценка, план спринта, статус.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="41.4" customHeight="1">
+      <c r="A4" s="200" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B4" s="200" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="C4" s="200" t="inlineStr">
+        <is>
+          <t>Область</t>
+        </is>
+      </c>
+      <c r="D4" s="200" t="inlineStr">
+        <is>
+          <t>Тип</t>
+        </is>
+      </c>
+      <c r="E4" s="200" t="inlineStr">
+        <is>
+          <t>Влияние</t>
+        </is>
+      </c>
+      <c r="F4" s="200" t="inlineStr">
+        <is>
+          <t>Оценка (дн)</t>
+        </is>
+      </c>
+      <c r="G4" s="200" t="inlineStr">
+        <is>
+          <t>Приоритет</t>
+        </is>
+      </c>
+      <c r="H4" s="200" t="inlineStr">
+        <is>
+          <t>Спринт</t>
+        </is>
+      </c>
+      <c r="I4" s="200" t="inlineStr">
+        <is>
+          <t>Статус</t>
+        </is>
+      </c>
+      <c r="J4" s="200" t="inlineStr">
+        <is>
+          <t>Спринт
+создан</t>
+        </is>
+      </c>
+      <c r="K4" s="200" t="inlineStr">
+        <is>
+          <t>Спринт
+погашен</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="27.6" customHeight="1">
+      <c r="A5" s="201" t="inlineStr">
+        <is>
+          <t>TD-1</t>
+        </is>
+      </c>
+      <c r="B5" s="202" t="inlineStr">
+        <is>
+          <t>Рефакторинг модуля авторизации</t>
+        </is>
+      </c>
+      <c r="C5" s="201" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="D5" s="201" t="inlineStr">
+        <is>
+          <t>Код</t>
+        </is>
+      </c>
+      <c r="E5" s="201" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F5" s="210" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" s="201" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H5" s="201" t="n">
+        <v>4</v>
+      </c>
+      <c r="I5" s="201" t="inlineStr">
+        <is>
+          <t>Закрыт</t>
+        </is>
+      </c>
+      <c r="J5" s="212" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="212" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" ht="27.6" customHeight="1">
+      <c r="A6" s="201" t="inlineStr">
+        <is>
+          <t>TD-2</t>
+        </is>
+      </c>
+      <c r="B6" s="202" t="inlineStr">
+        <is>
+          <t>Автотесты оформления заказа</t>
+        </is>
+      </c>
+      <c r="C6" s="201" t="inlineStr">
+        <is>
+          <t>Checkout</t>
+        </is>
+      </c>
+      <c r="D6" s="201" t="inlineStr">
+        <is>
+          <t>Тесты</t>
+        </is>
+      </c>
+      <c r="E6" s="201" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F6" s="210" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="201" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H6" s="201" t="n">
+        <v>3</v>
+      </c>
+      <c r="I6" s="201" t="inlineStr">
+        <is>
+          <t>Закрыт</t>
+        </is>
+      </c>
+      <c r="J6" s="212" t="n">
+        <v>2</v>
+      </c>
+      <c r="K6" s="212" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="201" t="inlineStr">
+        <is>
+          <t>TD-3</t>
+        </is>
+      </c>
+      <c r="B7" s="202" t="inlineStr">
+        <is>
+          <t>Убрать дубли в API заказов</t>
+        </is>
+      </c>
+      <c r="C7" s="201" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="D7" s="201" t="inlineStr">
+        <is>
+          <t>Архитектура</t>
+        </is>
+      </c>
+      <c r="E7" s="201" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F7" s="210" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="201" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H7" s="201" t="n">
+        <v>5</v>
+      </c>
+      <c r="I7" s="201" t="inlineStr">
+        <is>
+          <t>Открыт</t>
+        </is>
+      </c>
+      <c r="J7" s="212" t="n">
+        <v>3</v>
+      </c>
+      <c r="K7" s="212" t="n"/>
+    </row>
+    <row r="8" ht="27.6" customHeight="1">
+      <c r="A8" s="201" t="inlineStr">
+        <is>
+          <t>TD-4</t>
+        </is>
+      </c>
+      <c r="B8" s="202" t="inlineStr">
+        <is>
+          <t>Обновить документацию API</t>
+        </is>
+      </c>
+      <c r="C8" s="201" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="D8" s="201" t="inlineStr">
+        <is>
+          <t>Документация</t>
+        </is>
+      </c>
+      <c r="E8" s="201" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F8" s="210" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="201" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H8" s="201" t="n">
+        <v>6</v>
+      </c>
+      <c r="I8" s="201" t="inlineStr">
+        <is>
+          <t>Открыт</t>
+        </is>
+      </c>
+      <c r="J8" s="212" t="n">
+        <v>4</v>
+      </c>
+      <c r="K8" s="212" t="n"/>
+    </row>
+    <row r="9" ht="27.6" customHeight="1">
+      <c r="A9" s="201" t="inlineStr">
+        <is>
+          <t>TD-5</t>
+        </is>
+      </c>
+      <c r="B9" s="202" t="inlineStr">
+        <is>
+          <t>Мониторинг и алерты платежей</t>
+        </is>
+      </c>
+      <c r="C9" s="201" t="inlineStr">
+        <is>
+          <t>Payments</t>
+        </is>
+      </c>
+      <c r="D9" s="201" t="inlineStr">
+        <is>
+          <t>Инфраструктура</t>
+        </is>
+      </c>
+      <c r="E9" s="201" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F9" s="210" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="201" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H9" s="201" t="n">
+        <v>5</v>
+      </c>
+      <c r="I9" s="201" t="inlineStr">
+        <is>
+          <t>В работе</t>
+        </is>
+      </c>
+      <c r="J9" s="212" t="n">
+        <v>3</v>
+      </c>
+      <c r="K9" s="212" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="201" t="inlineStr">
+        <is>
+          <t>TD-6</t>
+        </is>
+      </c>
+      <c r="B10" s="202" t="inlineStr">
+        <is>
+          <t>Оптимизация запросов БД</t>
+        </is>
+      </c>
+      <c r="C10" s="201" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="D10" s="201" t="inlineStr">
+        <is>
+          <t>Код</t>
+        </is>
+      </c>
+      <c r="E10" s="201" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F10" s="210" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" s="201" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H10" s="201" t="n">
+        <v>7</v>
+      </c>
+      <c r="I10" s="201" t="inlineStr">
+        <is>
+          <t>Открыт</t>
+        </is>
+      </c>
+      <c r="J10" s="212" t="n">
+        <v>5</v>
+      </c>
+      <c r="K10" s="212" t="n"/>
+    </row>
+    <row r="12" ht="15.6" customHeight="1">
+      <c r="A12" s="207" t="inlineStr">
+        <is>
+          <t>По типу</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="200" t="inlineStr">
+        <is>
+          <t>Тип</t>
+        </is>
+      </c>
+      <c r="B13" s="200" t="inlineStr">
+        <is>
+          <t>Оценка (дн)</t>
+        </is>
+      </c>
+      <c r="C13" s="200" t="inlineStr">
+        <is>
+          <t>Кол-во</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="27.6" customHeight="1">
+      <c r="A14" s="208" t="inlineStr">
+        <is>
+          <t>Архитектура</t>
+        </is>
+      </c>
+      <c r="B14" s="206">
+        <f>SUMIF($D$5:$D$10,A14,$F$5:$F$10)</f>
+        <v/>
+      </c>
+      <c r="C14" s="205">
+        <f>COUNTIF($D$5:$D$10,A14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="208" t="inlineStr">
+        <is>
+          <t>Код</t>
+        </is>
+      </c>
+      <c r="B15" s="206">
+        <f>SUMIF($D$5:$D$10,A15,$F$5:$F$10)</f>
+        <v/>
+      </c>
+      <c r="C15" s="205">
+        <f>COUNTIF($D$5:$D$10,A15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="208" t="inlineStr">
+        <is>
+          <t>Тесты</t>
+        </is>
+      </c>
+      <c r="B16" s="206">
+        <f>SUMIF($D$5:$D$10,A16,$F$5:$F$10)</f>
+        <v/>
+      </c>
+      <c r="C16" s="205">
+        <f>COUNTIF($D$5:$D$10,A16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="208" t="inlineStr">
+        <is>
+          <t>Инфраструктура</t>
+        </is>
+      </c>
+      <c r="B17" s="206">
+        <f>SUMIF($D$5:$D$10,A17,$F$5:$F$10)</f>
+        <v/>
+      </c>
+      <c r="C17" s="205">
+        <f>COUNTIF($D$5:$D$10,A17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="208" t="inlineStr">
+        <is>
+          <t>Документация</t>
+        </is>
+      </c>
+      <c r="B18" s="206">
+        <f>SUMIF($D$5:$D$10,A18,$F$5:$F$10)</f>
+        <v/>
+      </c>
+      <c r="C18" s="205">
+        <f>COUNTIF($D$5:$D$10,A18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="15.6" customHeight="1">
+      <c r="A20" s="207" t="inlineStr">
+        <is>
+          <t>По статусу</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="200" t="inlineStr">
+        <is>
+          <t>Статус</t>
+        </is>
+      </c>
+      <c r="B21" s="200" t="inlineStr">
+        <is>
+          <t>Кол-во</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="208" t="inlineStr">
+        <is>
+          <t>Открыт</t>
+        </is>
+      </c>
+      <c r="B22" s="205">
+        <f>COUNTIF($I$5:$I$10,A22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="208" t="inlineStr">
+        <is>
+          <t>В работе</t>
+        </is>
+      </c>
+      <c r="B23" s="205">
+        <f>COUNTIF($I$5:$I$10,A23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="208" t="inlineStr">
+        <is>
+          <t>Закрыт</t>
+        </is>
+      </c>
+      <c r="B24" s="205">
+        <f>COUNTIF($I$5:$I$10,A24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="15.6" customHeight="1">
+      <c r="A27" s="207" t="inlineStr">
+        <is>
+          <t>Тренд техдолга (создано / погашено по спринтам)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="27.6" customHeight="1">
+      <c r="A28" s="200" t="inlineStr">
+        <is>
+          <t>Спринт</t>
+        </is>
+      </c>
+      <c r="B28" s="200" t="inlineStr">
+        <is>
+          <t>Создано</t>
+        </is>
+      </c>
+      <c r="C28" s="200" t="inlineStr">
+        <is>
+          <t>Погашено</t>
+        </is>
+      </c>
+      <c r="D28" s="200" t="inlineStr">
+        <is>
+          <t>Открыто (накопит.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="208" t="n">
+        <v>1</v>
+      </c>
+      <c r="B29" s="205">
+        <f>COUNTIF($J$5:$J$10,A29)</f>
+        <v/>
+      </c>
+      <c r="C29" s="205">
+        <f>COUNTIF($K$5:$K$10,A29)</f>
+        <v/>
+      </c>
+      <c r="D29" s="209">
+        <f>B29-C29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="208" t="n">
+        <v>2</v>
+      </c>
+      <c r="B30" s="205">
+        <f>COUNTIF($J$5:$J$10,A30)</f>
+        <v/>
+      </c>
+      <c r="C30" s="205">
+        <f>COUNTIF($K$5:$K$10,A30)</f>
+        <v/>
+      </c>
+      <c r="D30" s="209">
+        <f>D29+B30-C30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="208" t="n">
+        <v>3</v>
+      </c>
+      <c r="B31" s="205">
+        <f>COUNTIF($J$5:$J$10,A31)</f>
+        <v/>
+      </c>
+      <c r="C31" s="205">
+        <f>COUNTIF($K$5:$K$10,A31)</f>
+        <v/>
+      </c>
+      <c r="D31" s="209">
+        <f>D30+B31-C31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="208" t="n">
+        <v>4</v>
+      </c>
+      <c r="B32" s="205">
+        <f>COUNTIF($J$5:$J$10,A32)</f>
+        <v/>
+      </c>
+      <c r="C32" s="205">
+        <f>COUNTIF($K$5:$K$10,A32)</f>
+        <v/>
+      </c>
+      <c r="D32" s="209">
+        <f>D31+B32-C32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="208" t="n">
+        <v>5</v>
+      </c>
+      <c r="B33" s="205">
+        <f>COUNTIF($J$5:$J$10,A33)</f>
+        <v/>
+      </c>
+      <c r="C33" s="205">
+        <f>COUNTIF($K$5:$K$10,A33)</f>
+        <v/>
+      </c>
+      <c r="D33" s="209">
+        <f>D32+B33-C33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="208" t="n">
+        <v>6</v>
+      </c>
+      <c r="B34" s="205">
+        <f>COUNTIF($J$5:$J$10,A34)</f>
+        <v/>
+      </c>
+      <c r="C34" s="205">
+        <f>COUNTIF($K$5:$K$10,A34)</f>
+        <v/>
+      </c>
+      <c r="D34" s="209">
+        <f>D33+B34-C34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="208" t="n">
+        <v>7</v>
+      </c>
+      <c r="B35" s="205">
+        <f>COUNTIF($J$5:$J$10,A35)</f>
+        <v/>
+      </c>
+      <c r="C35" s="205">
+        <f>COUNTIF($K$5:$K$10,A35)</f>
+        <v/>
+      </c>
+      <c r="D35" s="209">
+        <f>D34+B35-C35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="208" t="n">
+        <v>8</v>
+      </c>
+      <c r="B36" s="205">
+        <f>COUNTIF($J$5:$J$10,A36)</f>
+        <v/>
+      </c>
+      <c r="C36" s="205">
+        <f>COUNTIF($K$5:$K$10,A36)</f>
+        <v/>
+      </c>
+      <c r="D36" s="209">
+        <f>D35+B36-C36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="208" t="n">
+        <v>9</v>
+      </c>
+      <c r="B37" s="205">
+        <f>COUNTIF($J$5:$J$10,A37)</f>
+        <v/>
+      </c>
+      <c r="C37" s="205">
+        <f>COUNTIF($K$5:$K$10,A37)</f>
+        <v/>
+      </c>
+      <c r="D37" s="209">
+        <f>D36+B37-C37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="208" t="n">
+        <v>10</v>
+      </c>
+      <c r="B38" s="205">
+        <f>COUNTIF($J$5:$J$10,A38)</f>
+        <v/>
+      </c>
+      <c r="C38" s="205">
+        <f>COUNTIF($K$5:$K$10,A38)</f>
+        <v/>
+      </c>
+      <c r="D38" s="209">
+        <f>D37+B38-C38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="208" t="n">
+        <v>11</v>
+      </c>
+      <c r="B39" s="205">
+        <f>COUNTIF($J$5:$J$10,A39)</f>
+        <v/>
+      </c>
+      <c r="C39" s="205">
+        <f>COUNTIF($K$5:$K$10,A39)</f>
+        <v/>
+      </c>
+      <c r="D39" s="209">
+        <f>D38+B39-C39</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="D5 D6 D7 D8 D9 D10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Архитектура,Код,Тесты,Инфраструктура,Документация"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E5 E6 E7 E8 E9 E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"High,Medium,Low"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I5 I6 I7 I8 I9 I10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Открыт,В работе,Закрыт"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
@@ -26079,7 +27024,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26469,7 +27414,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26711,7 +27656,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27067,7 +28012,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -28817,7 +29762,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -33719,7 +34664,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -33881,7 +34826,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -34538,7 +35483,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -37285,448 +38230,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D32"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="19.33203125" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="17.4" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Диаграмма сгорания (burndown) по задачам</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Идеальная линия — равномерное сгорание. Фактический остаток обновляется каждый день (жёлтый столбец).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>Всего работы тек. спринта (дн):</t>
-        </is>
-      </c>
-      <c r="B3" s="25">
-        <f>SUMIF(Бэклог!$M$5:$M$44,Параметры!$B$13,Бэклог!$E$5:$E$44)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>Рабочих дней:</t>
-        </is>
-      </c>
-      <c r="B4" s="15">
-        <f>SUMIF('Дорожная карта'!$A$6:$A$16,Параметры!$B$13,'Дорожная карта'!$E$6:$E$16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6" ht="27.6" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>День</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Дата</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Идеальный остаток (дн)</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Факт. остаток (дн)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="B7" s="22">
-        <f>WORKDAY(Параметры!$B$6,A7)</f>
-        <v/>
-      </c>
-      <c r="C7" s="23">
-        <f>$B$3*($B$4-A7)/$B$4</f>
-        <v/>
-      </c>
-      <c r="D7" s="24">
-        <f>$B$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B8" s="22">
-        <f>WORKDAY(Параметры!$B$6,A8)</f>
-        <v/>
-      </c>
-      <c r="C8" s="23">
-        <f>$B$3*($B$4-A8)/$B$4</f>
-        <v/>
-      </c>
-      <c r="D8" s="24">
-        <f>ROUND($B$3*0.98,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B9" s="22">
-        <f>WORKDAY(Параметры!$B$6,A9)</f>
-        <v/>
-      </c>
-      <c r="C9" s="23">
-        <f>$B$3*($B$4-A9)/$B$4</f>
-        <v/>
-      </c>
-      <c r="D9" s="24">
-        <f>ROUND($B$3*0.9,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B10" s="22">
-        <f>WORKDAY(Параметры!$B$6,A10)</f>
-        <v/>
-      </c>
-      <c r="C10" s="23">
-        <f>$B$3*($B$4-A10)/$B$4</f>
-        <v/>
-      </c>
-      <c r="D10" s="24">
-        <f>ROUND($B$3*0.86,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B11" s="22">
-        <f>WORKDAY(Параметры!$B$6,A11)</f>
-        <v/>
-      </c>
-      <c r="C11" s="23">
-        <f>$B$3*($B$4-A11)/$B$4</f>
-        <v/>
-      </c>
-      <c r="D11" s="24">
-        <f>ROUND($B$3*0.72,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B12" s="22">
-        <f>WORKDAY(Параметры!$B$6,A12)</f>
-        <v/>
-      </c>
-      <c r="C12" s="23">
-        <f>$B$3*($B$4-A12)/$B$4</f>
-        <v/>
-      </c>
-      <c r="D12" s="24">
-        <f>ROUND($B$3*0.6,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="B13" s="22">
-        <f>WORKDAY(Параметры!$B$6,A13)</f>
-        <v/>
-      </c>
-      <c r="C13" s="23">
-        <f>$B$3*($B$4-A13)/$B$4</f>
-        <v/>
-      </c>
-      <c r="D13" s="24">
-        <f>ROUND($B$3*0.55,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B14" s="22">
-        <f>WORKDAY(Параметры!$B$6,A14)</f>
-        <v/>
-      </c>
-      <c r="C14" s="23">
-        <f>$B$3*($B$4-A14)/$B$4</f>
-        <v/>
-      </c>
-      <c r="D14" s="24">
-        <f>ROUND($B$3*0.4,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B15" s="22">
-        <f>WORKDAY(Параметры!$B$6,A15)</f>
-        <v/>
-      </c>
-      <c r="C15" s="23">
-        <f>$B$3*($B$4-A15)/$B$4</f>
-        <v/>
-      </c>
-      <c r="D15" s="24">
-        <f>ROUND($B$3*0.28,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B16" s="22">
-        <f>WORKDAY(Параметры!$B$6,A16)</f>
-        <v/>
-      </c>
-      <c r="C16" s="23">
-        <f>$B$3*($B$4-A16)/$B$4</f>
-        <v/>
-      </c>
-      <c r="D16" s="24">
-        <f>ROUND($B$3*0.12,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="B17" s="22">
-        <f>WORKDAY(Параметры!$B$6,A17)</f>
-        <v/>
-      </c>
-      <c r="C17" s="23">
-        <f>$B$3*($B$4-A17)/$B$4</f>
-        <v/>
-      </c>
-      <c r="D17" s="24">
-        <f>ROUND($B$3*0,1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="14" t="inlineStr">
-        <is>
-          <t>Как читать:</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15.6" customHeight="1">
-      <c r="A20" s="91" t="inlineStr">
-        <is>
-          <t>Burn-up: объём vs накопленно сделано</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="41.4" customHeight="1">
-      <c r="A21" s="92" t="inlineStr">
-        <is>
-          <t>Спринт</t>
-        </is>
-      </c>
-      <c r="B21" s="92" t="inlineStr">
-        <is>
-          <t>Накопл.
-сделано (дн)</t>
-        </is>
-      </c>
-      <c r="C21" s="92" t="inlineStr">
-        <is>
-          <t>Общий
-объём (дн)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="110" t="n">
-        <v>1</v>
-      </c>
-      <c r="B22" s="102">
-        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A22)</f>
-        <v/>
-      </c>
-      <c r="C22" s="102">
-        <f>SUM(Бэклог!$E$5:$E$44)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="110" t="n">
-        <v>2</v>
-      </c>
-      <c r="B23" s="102">
-        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A23)</f>
-        <v/>
-      </c>
-      <c r="C23" s="102">
-        <f>SUM(Бэклог!$E$5:$E$44)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="110" t="n">
-        <v>3</v>
-      </c>
-      <c r="B24" s="102">
-        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A24)</f>
-        <v/>
-      </c>
-      <c r="C24" s="102">
-        <f>SUM(Бэклог!$E$5:$E$44)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="110" t="n">
-        <v>4</v>
-      </c>
-      <c r="B25" s="102">
-        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A25)</f>
-        <v/>
-      </c>
-      <c r="C25" s="102">
-        <f>SUM(Бэклог!$E$5:$E$44)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="110" t="n">
-        <v>5</v>
-      </c>
-      <c r="B26" s="102">
-        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A26)</f>
-        <v/>
-      </c>
-      <c r="C26" s="102">
-        <f>SUM(Бэклог!$E$5:$E$44)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="110" t="n">
-        <v>6</v>
-      </c>
-      <c r="B27" s="102">
-        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A27)</f>
-        <v/>
-      </c>
-      <c r="C27" s="102">
-        <f>SUM(Бэклог!$E$5:$E$44)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="110" t="n">
-        <v>7</v>
-      </c>
-      <c r="B28" s="102">
-        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A28)</f>
-        <v/>
-      </c>
-      <c r="C28" s="102">
-        <f>SUM(Бэклог!$E$5:$E$44)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="110" t="n">
-        <v>8</v>
-      </c>
-      <c r="B29" s="102">
-        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A29)</f>
-        <v/>
-      </c>
-      <c r="C29" s="102">
-        <f>SUM(Бэклог!$E$5:$E$44)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="110" t="n">
-        <v>9</v>
-      </c>
-      <c r="B30" s="102">
-        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A30)</f>
-        <v/>
-      </c>
-      <c r="C30" s="102">
-        <f>SUM(Бэклог!$E$5:$E$44)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="110" t="n">
-        <v>10</v>
-      </c>
-      <c r="B31" s="102">
-        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A31)</f>
-        <v/>
-      </c>
-      <c r="C31" s="102">
-        <f>SUM(Бэклог!$E$5:$E$44)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="110" t="n">
-        <v>11</v>
-      </c>
-      <c r="B32" s="102">
-        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A32)</f>
-        <v/>
-      </c>
-      <c r="C32" s="102">
-        <f>SUM(Бэклог!$E$5:$E$44)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -38169,6 +38672,448 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="19.33203125" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="17.4" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Диаграмма сгорания (burndown) по задачам</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Идеальная линия — равномерное сгорание. Фактический остаток обновляется каждый день (жёлтый столбец).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>Всего работы тек. спринта (дн):</t>
+        </is>
+      </c>
+      <c r="B3" s="25">
+        <f>SUMIF(Бэклог!$M$5:$M$44,Параметры!$B$13,Бэклог!$E$5:$E$44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Рабочих дней:</t>
+        </is>
+      </c>
+      <c r="B4" s="15">
+        <f>SUMIF('Дорожная карта'!$A$6:$A$16,Параметры!$B$13,'Дорожная карта'!$E$6:$E$16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="27.6" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>День</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Дата</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Идеальный остаток (дн)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Факт. остаток (дн)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="B7" s="22">
+        <f>WORKDAY(Параметры!$B$6,A7)</f>
+        <v/>
+      </c>
+      <c r="C7" s="23">
+        <f>$B$3*($B$4-A7)/$B$4</f>
+        <v/>
+      </c>
+      <c r="D7" s="24">
+        <f>$B$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="22">
+        <f>WORKDAY(Параметры!$B$6,A8)</f>
+        <v/>
+      </c>
+      <c r="C8" s="23">
+        <f>$B$3*($B$4-A8)/$B$4</f>
+        <v/>
+      </c>
+      <c r="D8" s="24">
+        <f>ROUND($B$3*0.98,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="22">
+        <f>WORKDAY(Параметры!$B$6,A9)</f>
+        <v/>
+      </c>
+      <c r="C9" s="23">
+        <f>$B$3*($B$4-A9)/$B$4</f>
+        <v/>
+      </c>
+      <c r="D9" s="24">
+        <f>ROUND($B$3*0.9,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="22">
+        <f>WORKDAY(Параметры!$B$6,A10)</f>
+        <v/>
+      </c>
+      <c r="C10" s="23">
+        <f>$B$3*($B$4-A10)/$B$4</f>
+        <v/>
+      </c>
+      <c r="D10" s="24">
+        <f>ROUND($B$3*0.86,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" s="22">
+        <f>WORKDAY(Параметры!$B$6,A11)</f>
+        <v/>
+      </c>
+      <c r="C11" s="23">
+        <f>$B$3*($B$4-A11)/$B$4</f>
+        <v/>
+      </c>
+      <c r="D11" s="24">
+        <f>ROUND($B$3*0.72,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" s="22">
+        <f>WORKDAY(Параметры!$B$6,A12)</f>
+        <v/>
+      </c>
+      <c r="C12" s="23">
+        <f>$B$3*($B$4-A12)/$B$4</f>
+        <v/>
+      </c>
+      <c r="D12" s="24">
+        <f>ROUND($B$3*0.6,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" s="22">
+        <f>WORKDAY(Параметры!$B$6,A13)</f>
+        <v/>
+      </c>
+      <c r="C13" s="23">
+        <f>$B$3*($B$4-A13)/$B$4</f>
+        <v/>
+      </c>
+      <c r="D13" s="24">
+        <f>ROUND($B$3*0.55,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B14" s="22">
+        <f>WORKDAY(Параметры!$B$6,A14)</f>
+        <v/>
+      </c>
+      <c r="C14" s="23">
+        <f>$B$3*($B$4-A14)/$B$4</f>
+        <v/>
+      </c>
+      <c r="D14" s="24">
+        <f>ROUND($B$3*0.4,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B15" s="22">
+        <f>WORKDAY(Параметры!$B$6,A15)</f>
+        <v/>
+      </c>
+      <c r="C15" s="23">
+        <f>$B$3*($B$4-A15)/$B$4</f>
+        <v/>
+      </c>
+      <c r="D15" s="24">
+        <f>ROUND($B$3*0.28,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="22">
+        <f>WORKDAY(Параметры!$B$6,A16)</f>
+        <v/>
+      </c>
+      <c r="C16" s="23">
+        <f>$B$3*($B$4-A16)/$B$4</f>
+        <v/>
+      </c>
+      <c r="D16" s="24">
+        <f>ROUND($B$3*0.12,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="B17" s="22">
+        <f>WORKDAY(Параметры!$B$6,A17)</f>
+        <v/>
+      </c>
+      <c r="C17" s="23">
+        <f>$B$3*($B$4-A17)/$B$4</f>
+        <v/>
+      </c>
+      <c r="D17" s="24">
+        <f>ROUND($B$3*0,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Как читать:</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15.6" customHeight="1">
+      <c r="A20" s="91" t="inlineStr">
+        <is>
+          <t>Burn-up: объём vs накопленно сделано</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="41.4" customHeight="1">
+      <c r="A21" s="92" t="inlineStr">
+        <is>
+          <t>Спринт</t>
+        </is>
+      </c>
+      <c r="B21" s="92" t="inlineStr">
+        <is>
+          <t>Накопл.
+сделано (дн)</t>
+        </is>
+      </c>
+      <c r="C21" s="92" t="inlineStr">
+        <is>
+          <t>Общий
+объём (дн)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="110" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" s="102">
+        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A22)</f>
+        <v/>
+      </c>
+      <c r="C22" s="102">
+        <f>SUM(Бэклог!$E$5:$E$44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="110" t="n">
+        <v>2</v>
+      </c>
+      <c r="B23" s="102">
+        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A23)</f>
+        <v/>
+      </c>
+      <c r="C23" s="102">
+        <f>SUM(Бэклог!$E$5:$E$44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="110" t="n">
+        <v>3</v>
+      </c>
+      <c r="B24" s="102">
+        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A24)</f>
+        <v/>
+      </c>
+      <c r="C24" s="102">
+        <f>SUM(Бэклог!$E$5:$E$44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="110" t="n">
+        <v>4</v>
+      </c>
+      <c r="B25" s="102">
+        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A25)</f>
+        <v/>
+      </c>
+      <c r="C25" s="102">
+        <f>SUM(Бэклог!$E$5:$E$44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="110" t="n">
+        <v>5</v>
+      </c>
+      <c r="B26" s="102">
+        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A26)</f>
+        <v/>
+      </c>
+      <c r="C26" s="102">
+        <f>SUM(Бэклог!$E$5:$E$44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="110" t="n">
+        <v>6</v>
+      </c>
+      <c r="B27" s="102">
+        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A27)</f>
+        <v/>
+      </c>
+      <c r="C27" s="102">
+        <f>SUM(Бэклог!$E$5:$E$44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="110" t="n">
+        <v>7</v>
+      </c>
+      <c r="B28" s="102">
+        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A28)</f>
+        <v/>
+      </c>
+      <c r="C28" s="102">
+        <f>SUM(Бэклог!$E$5:$E$44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="110" t="n">
+        <v>8</v>
+      </c>
+      <c r="B29" s="102">
+        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A29)</f>
+        <v/>
+      </c>
+      <c r="C29" s="102">
+        <f>SUM(Бэклог!$E$5:$E$44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="110" t="n">
+        <v>9</v>
+      </c>
+      <c r="B30" s="102">
+        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A30)</f>
+        <v/>
+      </c>
+      <c r="C30" s="102">
+        <f>SUM(Бэклог!$E$5:$E$44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="110" t="n">
+        <v>10</v>
+      </c>
+      <c r="B31" s="102">
+        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A31)</f>
+        <v/>
+      </c>
+      <c r="C31" s="102">
+        <f>SUM(Бэклог!$E$5:$E$44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="110" t="n">
+        <v>11</v>
+      </c>
+      <c r="B32" s="102">
+        <f>SUMIFS('Дорожная карта'!$I$6:$I$16,'Дорожная карта'!$A$6:$A$16,"&lt;="&amp;A32)</f>
+        <v/>
+      </c>
+      <c r="C32" s="102">
+        <f>SUM(Бэклог!$E$5:$E$44)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
@@ -38703,7 +39648,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -40259,7 +41204,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -40556,7 +41501,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -41302,7 +42247,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -41933,7 +42878,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -42194,7 +43139,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -42608,7 +43553,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -43103,7 +44048,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -46205,6 +47150,556 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="213" t="inlineStr">
+        <is>
+          <t>Оценка приоритетов по RICE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="229" t="inlineStr">
+        <is>
+          <t>RICE = (Reach × Impact × Confidence) / Effort. Чем выше балл — тем выше приоритет фичи.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="230" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B4" s="230" t="inlineStr">
+        <is>
+          <t>Фича / инициатива</t>
+        </is>
+      </c>
+      <c r="C4" s="230" t="inlineStr">
+        <is>
+          <t>Reach
+(польз./кв)</t>
+        </is>
+      </c>
+      <c r="D4" s="230" t="inlineStr">
+        <is>
+          <t>Impact
+(влияние)</t>
+        </is>
+      </c>
+      <c r="E4" s="230" t="inlineStr">
+        <is>
+          <t>Confidence
+(увер-ть)</t>
+        </is>
+      </c>
+      <c r="F4" s="230" t="inlineStr">
+        <is>
+          <t>Effort
+(чел-дни)</t>
+        </is>
+      </c>
+      <c r="G4" s="230" t="inlineStr">
+        <is>
+          <t>RICE
+score</t>
+        </is>
+      </c>
+      <c r="H4" s="230" t="inlineStr">
+        <is>
+          <t>Ранг</t>
+        </is>
+      </c>
+      <c r="I4" s="230" t="inlineStr">
+        <is>
+          <t>Приоритет</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="231" t="inlineStr">
+        <is>
+          <t>F-01</t>
+        </is>
+      </c>
+      <c r="B5" s="232" t="inlineStr">
+        <is>
+          <t>MVP оформления заказа</t>
+        </is>
+      </c>
+      <c r="C5" s="233" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D5" s="234" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="235" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="234" t="n">
+        <v>40</v>
+      </c>
+      <c r="G5" s="236">
+        <f>IFERROR(C5*D5*E5/F5,0)</f>
+        <v/>
+      </c>
+      <c r="H5" s="234">
+        <f>IF(G5="","",RANK(G5,$G$5:$G$14))</f>
+        <v/>
+      </c>
+      <c r="I5" s="237">
+        <f>IF(G5="","",IF(G5&gt;=0.6*MAX($G$5:$G$14),"Высокий",IF(G5&gt;=0.3*MAX($G$5:$G$14),"Средний","Низкий")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="231" t="inlineStr">
+        <is>
+          <t>F-02</t>
+        </is>
+      </c>
+      <c r="B6" s="232" t="inlineStr">
+        <is>
+          <t>Оплата картой</t>
+        </is>
+      </c>
+      <c r="C6" s="233" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D6" s="234" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" s="235" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F6" s="234" t="n">
+        <v>25</v>
+      </c>
+      <c r="G6" s="236">
+        <f>IFERROR(C6*D6*E6/F6,0)</f>
+        <v/>
+      </c>
+      <c r="H6" s="234">
+        <f>IF(G6="","",RANK(G6,$G$5:$G$14))</f>
+        <v/>
+      </c>
+      <c r="I6" s="237">
+        <f>IF(G6="","",IF(G6&gt;=0.6*MAX($G$5:$G$14),"Высокий",IF(G6&gt;=0.3*MAX($G$5:$G$14),"Средний","Низкий")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="231" t="inlineStr">
+        <is>
+          <t>F-03</t>
+        </is>
+      </c>
+      <c r="B7" s="232" t="inlineStr">
+        <is>
+          <t>Промокоды и скидки</t>
+        </is>
+      </c>
+      <c r="C7" s="233" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D7" s="234" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="235" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F7" s="234" t="n">
+        <v>12</v>
+      </c>
+      <c r="G7" s="236">
+        <f>IFERROR(C7*D7*E7/F7,0)</f>
+        <v/>
+      </c>
+      <c r="H7" s="234">
+        <f>IF(G7="","",RANK(G7,$G$5:$G$14))</f>
+        <v/>
+      </c>
+      <c r="I7" s="237">
+        <f>IF(G7="","",IF(G7&gt;=0.6*MAX($G$5:$G$14),"Высокий",IF(G7&gt;=0.3*MAX($G$5:$G$14),"Средний","Низкий")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="231" t="inlineStr">
+        <is>
+          <t>F-04</t>
+        </is>
+      </c>
+      <c r="B8" s="232" t="inlineStr">
+        <is>
+          <t>Уведомления (e-mail/push)</t>
+        </is>
+      </c>
+      <c r="C8" s="233" t="n">
+        <v>4000</v>
+      </c>
+      <c r="D8" s="234" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="235" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F8" s="234" t="n">
+        <v>15</v>
+      </c>
+      <c r="G8" s="236">
+        <f>IFERROR(C8*D8*E8/F8,0)</f>
+        <v/>
+      </c>
+      <c r="H8" s="234">
+        <f>IF(G8="","",RANK(G8,$G$5:$G$14))</f>
+        <v/>
+      </c>
+      <c r="I8" s="237">
+        <f>IF(G8="","",IF(G8&gt;=0.6*MAX($G$5:$G$14),"Высокий",IF(G8&gt;=0.3*MAX($G$5:$G$14),"Средний","Низкий")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="231" t="inlineStr">
+        <is>
+          <t>F-05</t>
+        </is>
+      </c>
+      <c r="B9" s="232" t="inlineStr">
+        <is>
+          <t>История заказов</t>
+        </is>
+      </c>
+      <c r="C9" s="233" t="n">
+        <v>3500</v>
+      </c>
+      <c r="D9" s="234" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E9" s="235" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="234" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" s="236">
+        <f>IFERROR(C9*D9*E9/F9,0)</f>
+        <v/>
+      </c>
+      <c r="H9" s="234">
+        <f>IF(G9="","",RANK(G9,$G$5:$G$14))</f>
+        <v/>
+      </c>
+      <c r="I9" s="237">
+        <f>IF(G9="","",IF(G9&gt;=0.6*MAX($G$5:$G$14),"Высокий",IF(G9&gt;=0.3*MAX($G$5:$G$14),"Средний","Низкий")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="231" t="inlineStr">
+        <is>
+          <t>F-06</t>
+        </is>
+      </c>
+      <c r="B10" s="232" t="inlineStr">
+        <is>
+          <t>Мобильная вёрстка</t>
+        </is>
+      </c>
+      <c r="C10" s="233" t="n">
+        <v>4500</v>
+      </c>
+      <c r="D10" s="234" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="235" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F10" s="234" t="n">
+        <v>20</v>
+      </c>
+      <c r="G10" s="236">
+        <f>IFERROR(C10*D10*E10/F10,0)</f>
+        <v/>
+      </c>
+      <c r="H10" s="234">
+        <f>IF(G10="","",RANK(G10,$G$5:$G$14))</f>
+        <v/>
+      </c>
+      <c r="I10" s="237">
+        <f>IF(G10="","",IF(G10&gt;=0.6*MAX($G$5:$G$14),"Высокий",IF(G10&gt;=0.3*MAX($G$5:$G$14),"Средний","Низкий")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="231" t="inlineStr">
+        <is>
+          <t>F-07</t>
+        </is>
+      </c>
+      <c r="B11" s="232" t="inlineStr">
+        <is>
+          <t>Личный кабинет</t>
+        </is>
+      </c>
+      <c r="C11" s="233" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D11" s="234" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="235" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F11" s="234" t="n">
+        <v>18</v>
+      </c>
+      <c r="G11" s="236">
+        <f>IFERROR(C11*D11*E11/F11,0)</f>
+        <v/>
+      </c>
+      <c r="H11" s="234">
+        <f>IF(G11="","",RANK(G11,$G$5:$G$14))</f>
+        <v/>
+      </c>
+      <c r="I11" s="237">
+        <f>IF(G11="","",IF(G11&gt;=0.6*MAX($G$5:$G$14),"Высокий",IF(G11&gt;=0.3*MAX($G$5:$G$14),"Средний","Низкий")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="231" t="inlineStr">
+        <is>
+          <t>F-08</t>
+        </is>
+      </c>
+      <c r="B12" s="232" t="inlineStr">
+        <is>
+          <t>Рекомендации товаров</t>
+        </is>
+      </c>
+      <c r="C12" s="233" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D12" s="234" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="235" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F12" s="234" t="n">
+        <v>22</v>
+      </c>
+      <c r="G12" s="236">
+        <f>IFERROR(C12*D12*E12/F12,0)</f>
+        <v/>
+      </c>
+      <c r="H12" s="234">
+        <f>IF(G12="","",RANK(G12,$G$5:$G$14))</f>
+        <v/>
+      </c>
+      <c r="I12" s="237">
+        <f>IF(G12="","",IF(G12&gt;=0.6*MAX($G$5:$G$14),"Высокий",IF(G12&gt;=0.3*MAX($G$5:$G$14),"Средний","Низкий")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="231" t="inlineStr">
+        <is>
+          <t>F-09</t>
+        </is>
+      </c>
+      <c r="B13" s="232" t="inlineStr">
+        <is>
+          <t>Экспорт отчётов</t>
+        </is>
+      </c>
+      <c r="C13" s="233" t="n">
+        <v>800</v>
+      </c>
+      <c r="D13" s="234" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E13" s="235" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F13" s="234" t="n">
+        <v>8</v>
+      </c>
+      <c r="G13" s="236">
+        <f>IFERROR(C13*D13*E13/F13,0)</f>
+        <v/>
+      </c>
+      <c r="H13" s="234">
+        <f>IF(G13="","",RANK(G13,$G$5:$G$14))</f>
+        <v/>
+      </c>
+      <c r="I13" s="237">
+        <f>IF(G13="","",IF(G13&gt;=0.6*MAX($G$5:$G$14),"Высокий",IF(G13&gt;=0.3*MAX($G$5:$G$14),"Средний","Низкий")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="231" t="inlineStr">
+        <is>
+          <t>F-10</t>
+        </is>
+      </c>
+      <c r="B14" s="232" t="inlineStr">
+        <is>
+          <t>Мультиязычность</t>
+        </is>
+      </c>
+      <c r="C14" s="233" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D14" s="234" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="235" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F14" s="234" t="n">
+        <v>30</v>
+      </c>
+      <c r="G14" s="236">
+        <f>IFERROR(C14*D14*E14/F14,0)</f>
+        <v/>
+      </c>
+      <c r="H14" s="234">
+        <f>IF(G14="","",RANK(G14,$G$5:$G$14))</f>
+        <v/>
+      </c>
+      <c r="I14" s="237">
+        <f>IF(G14="","",IF(G14&gt;=0.6*MAX($G$5:$G$14),"Высокий",IF(G14&gt;=0.3*MAX($G$5:$G$14),"Средний","Низкий")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="222" t="inlineStr">
+        <is>
+          <t>Шкалы оценки</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="238" t="inlineStr">
+        <is>
+          <t>Impact (влияние на пользователя):</t>
+        </is>
+      </c>
+      <c r="B17" s="239" t="inlineStr">
+        <is>
+          <t>3 — массивное · 2 — высокое · 1 — среднее · 0.5 — низкое · 0.25 — минимальное</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="238" t="inlineStr">
+        <is>
+          <t>Confidence (уверенность в оценке):</t>
+        </is>
+      </c>
+      <c r="B18" s="239" t="inlineStr">
+        <is>
+          <t>100% — высокая · 80% — средняя · 50% — низкая</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="238" t="inlineStr">
+        <is>
+          <t>Reach:</t>
+        </is>
+      </c>
+      <c r="B19" s="239" t="inlineStr">
+        <is>
+          <t>сколько пользователей затронет фича за квартал</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="238" t="inlineStr">
+        <is>
+          <t>Effort:</t>
+        </is>
+      </c>
+      <c r="B20" s="239" t="inlineStr">
+        <is>
+          <t>суммарные трудозатраты команды, человеко-дни</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="238" t="inlineStr">
+        <is>
+          <t>Приоритет:</t>
+        </is>
+      </c>
+      <c r="B21" s="239" t="inlineStr">
+        <is>
+          <t>Высокий ≥ 60% макс. балла · Средний ≥ 30% · иначе Низкий</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="I5:I14">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="39">
+      <formula>"Высокий"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="40">
+      <formula>"Средний"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="41">
+      <formula>"Низкий"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G5:G14">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="D5:D14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"3,2,1,0.5,0.25"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E5:E14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1,0.8,0.5"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
@@ -46662,7 +48157,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -46998,7 +48493,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -47300,769 +48795,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K39"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="16.6640625" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="10.77734375" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="17.4" customHeight="1">
-      <c r="A1" s="198" t="inlineStr">
-        <is>
-          <t>Технический долг</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="199" t="inlineStr">
-        <is>
-          <t>Реестр техдолга: область, тип, влияние, оценка, план спринта, статус.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="41.4" customHeight="1">
-      <c r="A4" s="200" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B4" s="200" t="inlineStr">
-        <is>
-          <t>Описание</t>
-        </is>
-      </c>
-      <c r="C4" s="200" t="inlineStr">
-        <is>
-          <t>Область</t>
-        </is>
-      </c>
-      <c r="D4" s="200" t="inlineStr">
-        <is>
-          <t>Тип</t>
-        </is>
-      </c>
-      <c r="E4" s="200" t="inlineStr">
-        <is>
-          <t>Влияние</t>
-        </is>
-      </c>
-      <c r="F4" s="200" t="inlineStr">
-        <is>
-          <t>Оценка (дн)</t>
-        </is>
-      </c>
-      <c r="G4" s="200" t="inlineStr">
-        <is>
-          <t>Приоритет</t>
-        </is>
-      </c>
-      <c r="H4" s="200" t="inlineStr">
-        <is>
-          <t>Спринт</t>
-        </is>
-      </c>
-      <c r="I4" s="200" t="inlineStr">
-        <is>
-          <t>Статус</t>
-        </is>
-      </c>
-      <c r="J4" s="200" t="inlineStr">
-        <is>
-          <t>Спринт
-создан</t>
-        </is>
-      </c>
-      <c r="K4" s="200" t="inlineStr">
-        <is>
-          <t>Спринт
-погашен</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="27.6" customHeight="1">
-      <c r="A5" s="201" t="inlineStr">
-        <is>
-          <t>TD-1</t>
-        </is>
-      </c>
-      <c r="B5" s="202" t="inlineStr">
-        <is>
-          <t>Рефакторинг модуля авторизации</t>
-        </is>
-      </c>
-      <c r="C5" s="201" t="inlineStr">
-        <is>
-          <t>Auth</t>
-        </is>
-      </c>
-      <c r="D5" s="201" t="inlineStr">
-        <is>
-          <t>Код</t>
-        </is>
-      </c>
-      <c r="E5" s="201" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F5" s="210" t="n">
-        <v>3</v>
-      </c>
-      <c r="G5" s="201" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H5" s="201" t="n">
-        <v>4</v>
-      </c>
-      <c r="I5" s="201" t="inlineStr">
-        <is>
-          <t>Закрыт</t>
-        </is>
-      </c>
-      <c r="J5" s="212" t="n">
-        <v>1</v>
-      </c>
-      <c r="K5" s="212" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" ht="27.6" customHeight="1">
-      <c r="A6" s="201" t="inlineStr">
-        <is>
-          <t>TD-2</t>
-        </is>
-      </c>
-      <c r="B6" s="202" t="inlineStr">
-        <is>
-          <t>Автотесты оформления заказа</t>
-        </is>
-      </c>
-      <c r="C6" s="201" t="inlineStr">
-        <is>
-          <t>Checkout</t>
-        </is>
-      </c>
-      <c r="D6" s="201" t="inlineStr">
-        <is>
-          <t>Тесты</t>
-        </is>
-      </c>
-      <c r="E6" s="201" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F6" s="210" t="n">
-        <v>2</v>
-      </c>
-      <c r="G6" s="201" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H6" s="201" t="n">
-        <v>3</v>
-      </c>
-      <c r="I6" s="201" t="inlineStr">
-        <is>
-          <t>Закрыт</t>
-        </is>
-      </c>
-      <c r="J6" s="212" t="n">
-        <v>2</v>
-      </c>
-      <c r="K6" s="212" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="201" t="inlineStr">
-        <is>
-          <t>TD-3</t>
-        </is>
-      </c>
-      <c r="B7" s="202" t="inlineStr">
-        <is>
-          <t>Убрать дубли в API заказов</t>
-        </is>
-      </c>
-      <c r="C7" s="201" t="inlineStr">
-        <is>
-          <t>API</t>
-        </is>
-      </c>
-      <c r="D7" s="201" t="inlineStr">
-        <is>
-          <t>Архитектура</t>
-        </is>
-      </c>
-      <c r="E7" s="201" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F7" s="210" t="n">
-        <v>2</v>
-      </c>
-      <c r="G7" s="201" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H7" s="201" t="n">
-        <v>5</v>
-      </c>
-      <c r="I7" s="201" t="inlineStr">
-        <is>
-          <t>Открыт</t>
-        </is>
-      </c>
-      <c r="J7" s="212" t="n">
-        <v>3</v>
-      </c>
-      <c r="K7" s="212" t="n"/>
-    </row>
-    <row r="8" ht="27.6" customHeight="1">
-      <c r="A8" s="201" t="inlineStr">
-        <is>
-          <t>TD-4</t>
-        </is>
-      </c>
-      <c r="B8" s="202" t="inlineStr">
-        <is>
-          <t>Обновить документацию API</t>
-        </is>
-      </c>
-      <c r="C8" s="201" t="inlineStr">
-        <is>
-          <t>Docs</t>
-        </is>
-      </c>
-      <c r="D8" s="201" t="inlineStr">
-        <is>
-          <t>Документация</t>
-        </is>
-      </c>
-      <c r="E8" s="201" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F8" s="210" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" s="201" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="H8" s="201" t="n">
-        <v>6</v>
-      </c>
-      <c r="I8" s="201" t="inlineStr">
-        <is>
-          <t>Открыт</t>
-        </is>
-      </c>
-      <c r="J8" s="212" t="n">
-        <v>4</v>
-      </c>
-      <c r="K8" s="212" t="n"/>
-    </row>
-    <row r="9" ht="27.6" customHeight="1">
-      <c r="A9" s="201" t="inlineStr">
-        <is>
-          <t>TD-5</t>
-        </is>
-      </c>
-      <c r="B9" s="202" t="inlineStr">
-        <is>
-          <t>Мониторинг и алерты платежей</t>
-        </is>
-      </c>
-      <c r="C9" s="201" t="inlineStr">
-        <is>
-          <t>Payments</t>
-        </is>
-      </c>
-      <c r="D9" s="201" t="inlineStr">
-        <is>
-          <t>Инфраструктура</t>
-        </is>
-      </c>
-      <c r="E9" s="201" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F9" s="210" t="n">
-        <v>2</v>
-      </c>
-      <c r="G9" s="201" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H9" s="201" t="n">
-        <v>5</v>
-      </c>
-      <c r="I9" s="201" t="inlineStr">
-        <is>
-          <t>В работе</t>
-        </is>
-      </c>
-      <c r="J9" s="212" t="n">
-        <v>3</v>
-      </c>
-      <c r="K9" s="212" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="201" t="inlineStr">
-        <is>
-          <t>TD-6</t>
-        </is>
-      </c>
-      <c r="B10" s="202" t="inlineStr">
-        <is>
-          <t>Оптимизация запросов БД</t>
-        </is>
-      </c>
-      <c r="C10" s="201" t="inlineStr">
-        <is>
-          <t>DB</t>
-        </is>
-      </c>
-      <c r="D10" s="201" t="inlineStr">
-        <is>
-          <t>Код</t>
-        </is>
-      </c>
-      <c r="E10" s="201" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="F10" s="210" t="n">
-        <v>3</v>
-      </c>
-      <c r="G10" s="201" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H10" s="201" t="n">
-        <v>7</v>
-      </c>
-      <c r="I10" s="201" t="inlineStr">
-        <is>
-          <t>Открыт</t>
-        </is>
-      </c>
-      <c r="J10" s="212" t="n">
-        <v>5</v>
-      </c>
-      <c r="K10" s="212" t="n"/>
-    </row>
-    <row r="12" ht="15.6" customHeight="1">
-      <c r="A12" s="207" t="inlineStr">
-        <is>
-          <t>По типу</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="200" t="inlineStr">
-        <is>
-          <t>Тип</t>
-        </is>
-      </c>
-      <c r="B13" s="200" t="inlineStr">
-        <is>
-          <t>Оценка (дн)</t>
-        </is>
-      </c>
-      <c r="C13" s="200" t="inlineStr">
-        <is>
-          <t>Кол-во</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="27.6" customHeight="1">
-      <c r="A14" s="208" t="inlineStr">
-        <is>
-          <t>Архитектура</t>
-        </is>
-      </c>
-      <c r="B14" s="206">
-        <f>SUMIF($D$5:$D$10,A14,$F$5:$F$10)</f>
-        <v/>
-      </c>
-      <c r="C14" s="205">
-        <f>COUNTIF($D$5:$D$10,A14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="208" t="inlineStr">
-        <is>
-          <t>Код</t>
-        </is>
-      </c>
-      <c r="B15" s="206">
-        <f>SUMIF($D$5:$D$10,A15,$F$5:$F$10)</f>
-        <v/>
-      </c>
-      <c r="C15" s="205">
-        <f>COUNTIF($D$5:$D$10,A15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="208" t="inlineStr">
-        <is>
-          <t>Тесты</t>
-        </is>
-      </c>
-      <c r="B16" s="206">
-        <f>SUMIF($D$5:$D$10,A16,$F$5:$F$10)</f>
-        <v/>
-      </c>
-      <c r="C16" s="205">
-        <f>COUNTIF($D$5:$D$10,A16)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="208" t="inlineStr">
-        <is>
-          <t>Инфраструктура</t>
-        </is>
-      </c>
-      <c r="B17" s="206">
-        <f>SUMIF($D$5:$D$10,A17,$F$5:$F$10)</f>
-        <v/>
-      </c>
-      <c r="C17" s="205">
-        <f>COUNTIF($D$5:$D$10,A17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="208" t="inlineStr">
-        <is>
-          <t>Документация</t>
-        </is>
-      </c>
-      <c r="B18" s="206">
-        <f>SUMIF($D$5:$D$10,A18,$F$5:$F$10)</f>
-        <v/>
-      </c>
-      <c r="C18" s="205">
-        <f>COUNTIF($D$5:$D$10,A18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="15.6" customHeight="1">
-      <c r="A20" s="207" t="inlineStr">
-        <is>
-          <t>По статусу</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="200" t="inlineStr">
-        <is>
-          <t>Статус</t>
-        </is>
-      </c>
-      <c r="B21" s="200" t="inlineStr">
-        <is>
-          <t>Кол-во</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="208" t="inlineStr">
-        <is>
-          <t>Открыт</t>
-        </is>
-      </c>
-      <c r="B22" s="205">
-        <f>COUNTIF($I$5:$I$10,A22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="208" t="inlineStr">
-        <is>
-          <t>В работе</t>
-        </is>
-      </c>
-      <c r="B23" s="205">
-        <f>COUNTIF($I$5:$I$10,A23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="208" t="inlineStr">
-        <is>
-          <t>Закрыт</t>
-        </is>
-      </c>
-      <c r="B24" s="205">
-        <f>COUNTIF($I$5:$I$10,A24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="15.6" customHeight="1">
-      <c r="A27" s="207" t="inlineStr">
-        <is>
-          <t>Тренд техдолга (создано / погашено по спринтам)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="27.6" customHeight="1">
-      <c r="A28" s="200" t="inlineStr">
-        <is>
-          <t>Спринт</t>
-        </is>
-      </c>
-      <c r="B28" s="200" t="inlineStr">
-        <is>
-          <t>Создано</t>
-        </is>
-      </c>
-      <c r="C28" s="200" t="inlineStr">
-        <is>
-          <t>Погашено</t>
-        </is>
-      </c>
-      <c r="D28" s="200" t="inlineStr">
-        <is>
-          <t>Открыто (накопит.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="208" t="n">
-        <v>1</v>
-      </c>
-      <c r="B29" s="205">
-        <f>COUNTIF($J$5:$J$10,A29)</f>
-        <v/>
-      </c>
-      <c r="C29" s="205">
-        <f>COUNTIF($K$5:$K$10,A29)</f>
-        <v/>
-      </c>
-      <c r="D29" s="209">
-        <f>B29-C29</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="208" t="n">
-        <v>2</v>
-      </c>
-      <c r="B30" s="205">
-        <f>COUNTIF($J$5:$J$10,A30)</f>
-        <v/>
-      </c>
-      <c r="C30" s="205">
-        <f>COUNTIF($K$5:$K$10,A30)</f>
-        <v/>
-      </c>
-      <c r="D30" s="209">
-        <f>D29+B30-C30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="208" t="n">
-        <v>3</v>
-      </c>
-      <c r="B31" s="205">
-        <f>COUNTIF($J$5:$J$10,A31)</f>
-        <v/>
-      </c>
-      <c r="C31" s="205">
-        <f>COUNTIF($K$5:$K$10,A31)</f>
-        <v/>
-      </c>
-      <c r="D31" s="209">
-        <f>D30+B31-C31</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="208" t="n">
-        <v>4</v>
-      </c>
-      <c r="B32" s="205">
-        <f>COUNTIF($J$5:$J$10,A32)</f>
-        <v/>
-      </c>
-      <c r="C32" s="205">
-        <f>COUNTIF($K$5:$K$10,A32)</f>
-        <v/>
-      </c>
-      <c r="D32" s="209">
-        <f>D31+B32-C32</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="208" t="n">
-        <v>5</v>
-      </c>
-      <c r="B33" s="205">
-        <f>COUNTIF($J$5:$J$10,A33)</f>
-        <v/>
-      </c>
-      <c r="C33" s="205">
-        <f>COUNTIF($K$5:$K$10,A33)</f>
-        <v/>
-      </c>
-      <c r="D33" s="209">
-        <f>D32+B33-C33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="208" t="n">
-        <v>6</v>
-      </c>
-      <c r="B34" s="205">
-        <f>COUNTIF($J$5:$J$10,A34)</f>
-        <v/>
-      </c>
-      <c r="C34" s="205">
-        <f>COUNTIF($K$5:$K$10,A34)</f>
-        <v/>
-      </c>
-      <c r="D34" s="209">
-        <f>D33+B34-C34</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="208" t="n">
-        <v>7</v>
-      </c>
-      <c r="B35" s="205">
-        <f>COUNTIF($J$5:$J$10,A35)</f>
-        <v/>
-      </c>
-      <c r="C35" s="205">
-        <f>COUNTIF($K$5:$K$10,A35)</f>
-        <v/>
-      </c>
-      <c r="D35" s="209">
-        <f>D34+B35-C35</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="208" t="n">
-        <v>8</v>
-      </c>
-      <c r="B36" s="205">
-        <f>COUNTIF($J$5:$J$10,A36)</f>
-        <v/>
-      </c>
-      <c r="C36" s="205">
-        <f>COUNTIF($K$5:$K$10,A36)</f>
-        <v/>
-      </c>
-      <c r="D36" s="209">
-        <f>D35+B36-C36</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="208" t="n">
-        <v>9</v>
-      </c>
-      <c r="B37" s="205">
-        <f>COUNTIF($J$5:$J$10,A37)</f>
-        <v/>
-      </c>
-      <c r="C37" s="205">
-        <f>COUNTIF($K$5:$K$10,A37)</f>
-        <v/>
-      </c>
-      <c r="D37" s="209">
-        <f>D36+B37-C37</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="208" t="n">
-        <v>10</v>
-      </c>
-      <c r="B38" s="205">
-        <f>COUNTIF($J$5:$J$10,A38)</f>
-        <v/>
-      </c>
-      <c r="C38" s="205">
-        <f>COUNTIF($K$5:$K$10,A38)</f>
-        <v/>
-      </c>
-      <c r="D38" s="209">
-        <f>D37+B38-C38</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="208" t="n">
-        <v>11</v>
-      </c>
-      <c r="B39" s="205">
-        <f>COUNTIF($J$5:$J$10,A39)</f>
-        <v/>
-      </c>
-      <c r="C39" s="205">
-        <f>COUNTIF($K$5:$K$10,A39)</f>
-        <v/>
-      </c>
-      <c r="D39" s="209">
-        <f>D38+B39-C39</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="3">
-    <dataValidation sqref="D5 D6 D7 D8 D9 D10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Архитектура,Код,Тесты,Инфраструктура,Документация"</formula1>
-    </dataValidation>
-    <dataValidation sqref="E5 E6 E7 E8 E9 E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"High,Medium,Low"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I5 I6 I7 I8 I9 I10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Открыт,В работе,Закрыт"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>